<commit_message>
feat: Generate new application requirements and evaluation outputs by updating extraction and evaluation scripts, configuration, and ground truth data.
</commit_message>
<xml_diff>
--- a/ground_truth/bbmsa_ground_truth.xlsx
+++ b/ground_truth/bbmsa_ground_truth.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -448,290 +448,290 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>BBMSA-REQ-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Catalog Consolidation</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Migrate all relevant offerings to primary MCD catalog and decommission legacy catalogs (mx_DATAVALET, mx_MANAGED LAN, mx_MANAGED WAN, mx_MIS). Standardize on NSMIS service group.</t>
-        </is>
-      </c>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-002</t>
+          <t>BBMSA-REQ-001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Datavalet Meraki Wi-Fi Taxonomy</t>
+          <t>Catalog Consolidation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Reorganize Meraki Wi-Fi offerings under path: Managed Services -&gt; Bell Managed Services for Cisco Meraki -&gt; Wi-fi. Include all Datavalet Meraki Wi-Fi offerings.</t>
+          <t>Migrate all relevant offerings to primary MCD catalog and decommission legacy catalogs (mx_DATAVALET, mx_MANAGED LAN, mx_MANAGED WAN, mx_MIS). Standardize on NSMIS service group.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-003</t>
+          <t>BBMSA-REQ-002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Datavalet MIS Battery Taxonomy</t>
+          <t>Datavalet Meraki Wi-Fi Taxonomy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Reorganize MIS Battery offerings under path: Managed Services -&gt; Managed Infrastructure Services -&gt; Power supplies or battery backup.</t>
+          <t>Reorganize Meraki Wi-Fi offerings under path: Managed Services -&gt; Bell Managed Services for Cisco Meraki -&gt; Wi-fi. Include all Datavalet Meraki Wi-Fi offerings.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-004</t>
+          <t>BBMSA-REQ-003</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CI Filtering for Datavalet Offerings</t>
+          <t>Datavalet MIS Battery Taxonomy</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Datavalet offerings must ONLY show on CI selection page if device is managed by DATAVALET. Implement global filter to prevent Bell-managed devices from appearing.</t>
+          <t>Reorganize MIS Battery offerings under path: Managed Services -&gt; Managed Infrastructure Services -&gt; Power supplies or battery backup.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-005</t>
+          <t>BBMSA-REQ-004</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bell Managed Meraki Catalog Inclusion</t>
+          <t>CI Filtering for Datavalet Offerings</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Add Meraki offerings from Managed WAN and Managed LAN to MCD catalog. Exclude MERAKI_113. Implement global filter to hide Bell offerings if device managed by DATAVALET.</t>
+          <t>Datavalet offerings must ONLY show on CI selection page if device is managed by DATAVALET. Implement global filter to prevent Bell-managed devices from appearing.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-006</t>
+          <t>BBMSA-REQ-005</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Datavalet Transfer Site to Template (MCDO-03)</t>
+          <t>Bell Managed Meraki Catalog Inclusion</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Enable 'Transfer site to another template (profile)' action under Meraki Wi-fi -&gt; Modify. Show only Datavalet-managed CIs. Include mandatory dropdown for template selection. Rate Category 1.</t>
+          <t>Add Meraki offerings from Managed WAN and Managed LAN to MCD catalog. Exclude MERAKI_113. Implement global filter to hide Bell offerings if device managed by DATAVALET.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-007</t>
+          <t>BBMSA-REQ-006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bell Meraki Profile Modification (MCDO-01)</t>
+          <t>Datavalet Transfer Site to Template (MCDO-03)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Enable modification of Bell-managed Meraki profiles with new classification 41200340. Enable auto-creation of Change requests and flow-through. Rate Category Type 1.</t>
+          <t>Enable 'Transfer site to another template (profile)' action under Meraki Wi-fi -&gt; Modify. Show only Datavalet-managed CIs. Include mandatory dropdown for template selection. Rate Category 1.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-008</t>
+          <t>BBMSA-REQ-007</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Datavalet Create New Profile/Template (MCDO-04)</t>
+          <t>Bell Meraki Profile Modification (MCDO-01)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Enable 'Create new profile/template' action under Meraki Wi-fi -&gt; Add. Updated to Rate Category 3. Technical Details page must support custom payload definitions.</t>
+          <t>Enable modification of Bell-managed Meraki profiles with new classification 41200340. Enable auto-creation of Change requests and flow-through. Rate Category Type 1.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-009</t>
+          <t>BBMSA-REQ-008</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bell Create New Profile</t>
+          <t>Datavalet Create New Profile/Template (MCDO-04)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Enable Bell version of create new profile following Bell internal provisioning logic and Maximo job plans.</t>
+          <t>Enable 'Create new profile/template' action under Meraki Wi-fi -&gt; Add. Updated to Rate Category 3. Technical Details page must support custom payload definitions.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-010</t>
+          <t>BBMSA-REQ-009</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Maximo to ServiceNow Integration</t>
+          <t>Bell Create New Profile</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Implement REST API synchronization between Maximo and Datavalet ServiceNow. Sync SR creation, status updates, and field mappings without data truncation.</t>
+          <t>Enable Bell version of create new profile following Bell internal provisioning logic and Maximo job plans.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-011</t>
+          <t>BBMSA-REQ-010</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Offering Name Adjustments</t>
+          <t>Maximo to ServiceNow Integration</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Update DV-047 display name to 'Ad Hoc report or dashboard customization'. Remove 'an URL' and 'un URL' terminology from MERAKI_113 description.</t>
+          <t>Implement REST API synchronization between Maximo and Datavalet ServiceNow. Sync SR creation, status updates, and field mappings without data truncation.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-012</t>
+          <t>BBMSA-REQ-011</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CI Visibility Matrix</t>
+          <t>Offering Name Adjustments</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Implement CI visibility rules: Datavalet offerings visible only for DATAVALET-managed CIs, Bell offerings visible only for BELL-managed CIs. Support positive and negative test scenarios.</t>
+          <t>Update DV-047 display name to 'Ad Hoc report or dashboard customization'. Remove 'an URL' and 'un URL' terminology from MERAKI_113 description.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-013</t>
+          <t>BBMSA-REQ-012</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MACD Process Workflows</t>
+          <t>CI Visibility Matrix</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Implement three workflow types: Standard Selection (CI -&gt; Form -&gt; Submit), Redirected Selection (Modify -&gt; Template dropdown -&gt; Submit), External Sync (Maximo External Ticket -&gt; ServiceNow sync).</t>
+          <t>Implement CI visibility rules: Datavalet offerings visible only for DATAVALET-managed CIs, Bell offerings visible only for BELL-managed CIs. Support positive and negative test scenarios.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-014</t>
+          <t>BBMSA-REQ-013</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CI Selection Page UI</t>
+          <t>MACD Process Workflows</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Display CI selection page with filtering by device manager (DATAVALET or BELL). Include form fields for CI selection and technical details.</t>
+          <t>Implement three workflow types: Standard Selection (CI -&gt; Form -&gt; Submit), Redirected Selection (Modify -&gt; Template dropdown -&gt; Submit), External Sync (Maximo External Ticket -&gt; ServiceNow sync).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-015</t>
+          <t>BBMSA-REQ-014</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Technical Details Page UI</t>
+          <t>CI Selection Page UI</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Display technical details page with mandatory dropdown for template/profile selection. Support variable payload definitions for custom configurations.</t>
+          <t>Display CI selection page with filtering by device manager (DATAVALET or BELL). Include form fields for CI selection and technical details.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BBMSA-REQ-016</t>
+          <t>BBMSA-REQ-015</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Defect Prevention - CI Visibility</t>
+          <t>Technical Details Page UI</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Prevent regression of defects SADRSTRANG-13583 (CIs not appearing), OMNITOTORO-665 (wrong manager CIs appearing), OMNITOTORO-587 (service-unavailable errors).</t>
+          <t>Display technical details page with mandatory dropdown for template/profile selection. Support variable payload definitions for custom configurations.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>BBMSA-REQ-016</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Defect Prevention - CI Visibility</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Prevent regression of defects SADRSTRANG-13583 (CIs not appearing), OMNITOTORO-665 (wrong manager CIs appearing), OMNITOTORO-587 (service-unavailable errors).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>BBMSA-REQ-017</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Defect Prevention - Integration</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Prevent regression of defects SADRSTRANG-13420 (status sync failure), SADRSTRANG-13593 (incorrect payload on hold), SADEFENDER-373 (classification mismatch).</t>
         </is>

</xml_diff>